<commit_message>
Replace show notes card with Column E HTML content
</commit_message>
<xml_diff>
--- a/Movie Archive Inputs.xlsx
+++ b/Movie Archive Inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E65165-62A4-4188-BB7C-56029849ADF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A11AB435-A7A4-42DF-BD98-EE62D6A119C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,24 +17,18 @@
     <sheet name="Transcripts" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Movie Ratings'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Movie Ratings'!$A$1:$F$37</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="147">
   <si>
     <t>12 Angry Men</t>
   </si>
   <si>
-    <t>Did the prosecution actually prove the case?</t>
-  </si>
-  <si>
-    <t>Justice; civic duty; bias; memory; reasonable doubt</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=WjvBorOaAQc</t>
   </si>
   <si>
@@ -44,315 +38,105 @@
     <t>Arrival</t>
   </si>
   <si>
-    <t>If you could press a button and see the rest of your life, would you want to know?</t>
-  </si>
-  <si>
-    <t>Fate; language; love; grief; randomness; choice</t>
-  </si>
-  <si>
     <t>Baby Driver</t>
   </si>
   <si>
-    <t>What song did this movie remind you of?</t>
-  </si>
-  <si>
-    <t>Music; crime; technology aging</t>
-  </si>
-  <si>
     <t>Backrooms</t>
   </si>
   <si>
-    <t>Why did this movie become popular when the hosts found almost no story, character development, or payoff?</t>
-  </si>
-  <si>
-    <t>Isolation; loneliness; mental health; liminal spaces; identity; meaning-making; storytelling versus concept</t>
-  </si>
-  <si>
     <t>B.A.P.S.</t>
   </si>
   <si>
-    <t>What hybrid business would we open with our podcast studio?</t>
-  </si>
-  <si>
-    <t>90s comedy; class; fish-out-of-water; friendship; hood classics</t>
-  </si>
-  <si>
     <t>The Best Man</t>
   </si>
   <si>
-    <t>Does a secret like that ever truly stay buried?</t>
-  </si>
-  <si>
-    <t>Friendship; loyalty; betrayal</t>
-  </si>
-  <si>
     <t>Boomerang</t>
   </si>
   <si>
-    <t>Is this movie good?</t>
-  </si>
-  <si>
-    <t>Dating; ego; image</t>
-  </si>
-  <si>
     <t>Brown Sugar</t>
   </si>
   <si>
-    <t>When did you fall in love with hip-hop?</t>
-  </si>
-  <si>
-    <t>Hip-hop; friendship; love</t>
-  </si>
-  <si>
     <t>Children of Men</t>
   </si>
   <si>
-    <t>Do you have a go bag?</t>
-  </si>
-  <si>
-    <t>Collapse; infrastructure; survival</t>
-  </si>
-  <si>
     <t>The Dark Knight</t>
   </si>
   <si>
-    <t>Was Gotham better off preserving Harvey Dent's heroic image, even if it required lying to the public?</t>
-  </si>
-  <si>
-    <t>Order vs. chaos; burden of heroism; moral compromise; public faith and symbolism; law versus vigilantism; fragility of civilization; sacrifice</t>
-  </si>
-  <si>
     <t>Friday</t>
   </si>
   <si>
-    <t>Is Pineapple Express the white Friday?</t>
-  </si>
-  <si>
-    <t>Neighborhood; comedy; friendship</t>
-  </si>
-  <si>
     <t>Game Night</t>
   </si>
   <si>
-    <t>If you had a house in the suburbs, would you host?</t>
-  </si>
-  <si>
-    <t>Hosting; games; suburbs</t>
-  </si>
-  <si>
     <t>Good Boys</t>
   </si>
   <si>
-    <t>Are you still cool with anyone from grade school?</t>
-  </si>
-  <si>
-    <t>Childhood; friendship; growing up</t>
-  </si>
-  <si>
     <t>The Judge</t>
   </si>
   <si>
-    <t>Was the bathroom scene the most powerful scene?</t>
-  </si>
-  <si>
-    <t>Family; fathers; courtrooms</t>
-  </si>
-  <si>
     <t>Juror No. 2</t>
   </si>
   <si>
-    <t>What does justice require when protecting yourself could condemn someone else?</t>
-  </si>
-  <si>
-    <t>Justice; conscience; self-preservation</t>
-  </si>
-  <si>
     <t>Love &amp; Basketball</t>
   </si>
   <si>
-    <t>Was Monica wrong for leaving because of curfew?</t>
-  </si>
-  <si>
-    <t>Love; ambition; family; sports</t>
-  </si>
-  <si>
     <t>Love Jones</t>
   </si>
   <si>
-    <t>Was Darius who Nina wanted, or who was there when she was tired?</t>
-  </si>
-  <si>
-    <t>Romance; art; timing</t>
-  </si>
-  <si>
     <t>Mrs. Doubtfire</t>
   </si>
   <si>
-    <t>Did this movie age well?</t>
-  </si>
-  <si>
-    <t>Divorce; parenting; nostalgia</t>
-  </si>
-  <si>
     <t>Nick &amp; Norah's Infinite Playlist</t>
   </si>
   <si>
-    <t>What five acts would you do anything to see live?</t>
-  </si>
-  <si>
-    <t>Music; NYC; dating</t>
-  </si>
-  <si>
     <t>Obsession</t>
   </si>
   <si>
-    <t>Does unrequited love count as real love if it is never returned?</t>
-  </si>
-  <si>
-    <t>Be careful what you wish for; agency and coercion; unrequited love; attachment; youthful insecurity; control versus genuine affection</t>
-  </si>
-  <si>
     <t>The Odyssey</t>
   </si>
   <si>
-    <t>Is this Matt Damon's best role?</t>
-  </si>
-  <si>
-    <t>Journey; mythology; war; homecoming</t>
-  </si>
-  <si>
     <t>The Prestige</t>
   </si>
   <si>
-    <t>Did Borden tie the wrong knot, and did Borden truly know which knot was tied?</t>
-  </si>
-  <si>
-    <t>Obsession; sacrifice; rivalry; identity; showmanship versus craft; passion; deception; divided lives; the cost of applause</t>
-  </si>
-  <si>
     <t>Reservoir Dogs</t>
   </si>
   <si>
-    <t>Is Reservoir Dogs actually a great movie, or has its reputation been elevated because Tarantino later became one of the most acclaimed directors of all time?</t>
-  </si>
-  <si>
-    <t>Trust vs. self-preservation; loyalty and betrayal; the psychology of lying; reputation versus reality; criminal organizations; group dynamics under pressure; the costs of paranoia</t>
-  </si>
-  <si>
     <t>The Sandlot</t>
   </si>
   <si>
-    <t>Are you still friends with anyone from your childhood neighborhood?</t>
-  </si>
-  <si>
-    <t>Childhood; friendship; nostalgia</t>
-  </si>
-  <si>
     <t>Sleepy Hollow</t>
   </si>
   <si>
-    <t>Would you rather be the writer or director?</t>
-  </si>
-  <si>
-    <t>Mystery; supernatural; worldbuilding</t>
-  </si>
-  <si>
     <t>State Property</t>
   </si>
   <si>
-    <t>Was this the OG Tubi movie?</t>
-  </si>
-  <si>
-    <t>Nostalgia; crime; rap culture</t>
-  </si>
-  <si>
     <t>Still Alice</t>
   </si>
   <si>
-    <t>Would you use genetic testing to edit chronic illness out?</t>
-  </si>
-  <si>
-    <t>Memory; identity; illness</t>
-  </si>
-  <si>
     <t>Stranger Than Fiction</t>
   </si>
   <si>
-    <t>If a voice narrated your life, what genre would it be?</t>
-  </si>
-  <si>
-    <t>Routine; mortality; originality</t>
-  </si>
-  <si>
     <t>Take Me Home Tonight</t>
   </si>
   <si>
-    <t>What was your favorite Grand Theft Auto?</t>
-  </si>
-  <si>
-    <t>Adulthood; nostalgia; pressure</t>
-  </si>
-  <si>
     <t>The Drama</t>
   </si>
   <si>
-    <t>Is Emma's revelation alone enough to call off the wedding, or is the larger issue everything else surrounding her character?</t>
-  </si>
-  <si>
-    <t>Forgiveness; trust; hidden identity; mental health; love versus judgment; emotional immaturity; second chances; relationship pressure</t>
-  </si>
-  <si>
     <t>The Photograph</t>
   </si>
   <si>
-    <t>Should Michael have pursued a serious relationship with Mae while actively preparing to take a job in another country?</t>
-  </si>
-  <si>
-    <t>Family legacy; motherhood; generational trauma; ambition versus relationships; memory and grief; love across generations; identity and self-discovery</t>
-  </si>
-  <si>
     <t>This Christmas</t>
   </si>
   <si>
-    <t>Does your family do a big Christmas?</t>
-  </si>
-  <si>
-    <t>Family; holidays; secrets</t>
-  </si>
-  <si>
     <t>Weapons</t>
   </si>
   <si>
-    <t>Why did no one have guns?</t>
-  </si>
-  <si>
-    <t>Grief; suspense; endings</t>
-  </si>
-  <si>
     <t>White Men Can't Jump</t>
   </si>
   <si>
-    <t>Was Gloria right to leave?</t>
-  </si>
-  <si>
-    <t>Money; relationships; basketball</t>
-  </si>
-  <si>
     <t>You're Next</t>
   </si>
   <si>
-    <t>Why is everyone doing a contract killing the hard way?</t>
-  </si>
-  <si>
-    <t>Horror logic; survival; Halloween</t>
-  </si>
-  <si>
-    <t>How did this win Best Picture?</t>
-  </si>
-  <si>
-    <t>Aging; suburbia; discomfort; midlife crisis; adult rewatch</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=uVc5pvyebG8</t>
   </si>
   <si>
@@ -459,12 +243,6 @@
   </si>
   <si>
     <t>darius_rating</t>
-  </si>
-  <si>
-    <t>best_question</t>
-  </si>
-  <si>
-    <t>major_themes</t>
   </si>
   <si>
     <t>youtube_link</t>
@@ -6069,6 +5847,1069 @@
 Darius: ***** out. That's the whole point of why we are outside on Halloween.
 Jordan: This is literally the point of</t>
   </si>
+  <si>
+    <t>Show Notes &amp; Highlights</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Small Talk, WOOM, Sports section, and MY NOTES included Most elitist opinion, Aging, Does rewatchability matter, Pool Season, date contact, Rock Bottom, and similar prompts.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Courtroom drama about twelve jurors debating whether the state proved a murder case beyond a reasonable doubt.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act I: The Lone Voice — one juror forces the room to actually deliberate.&lt;/li&gt;
+    &lt;li&gt;Act II: Shifting the Tide — witness testimony, memory, bias, and burden of proof are challenged.&lt;/li&gt;
+    &lt;li&gt;Act III: The Final Verdict — the remaining holdouts confront their own reasoning.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Did the prosecution actually prove the case?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; It is not the defense’s job to prove innocence; it is the prosecution’s job to prove guilt.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Beyond a reasonable doubt should be a high burden before the state takes freedom.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Justice&lt;/li&gt;
+      &lt;li&gt;civic duty&lt;/li&gt;
+      &lt;li&gt;bias&lt;/li&gt;
+      &lt;li&gt;memory&lt;/li&gt;
+      &lt;li&gt;reasonable doubt&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Suburban midlife crisis drama about Lester Burnham rejecting his numb routine while the neighborhood’s secrets unravel.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act I: The Wake-Up Call — Lester’s routine breaks.&lt;/li&gt;
+    &lt;li&gt;Act II: Breaking the Mold — Lester rebels while the family fractures.&lt;/li&gt;
+    &lt;li&gt;Act III: The Beautiful End — the movie reaches its uncomfortable conclusion.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; How did this win Best Picture?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; It was not attraction; it was what youth represented.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Add this to the list of 90s movies about bored suburbanites who were too comfortable.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Aging&lt;/li&gt;
+      &lt;li&gt;suburbia&lt;/li&gt;
+      &lt;li&gt;discomfort&lt;/li&gt;
+      &lt;li&gt;midlife crisis&lt;/li&gt;
+      &lt;li&gt;adult rewatch&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;No original rundown captured in this import package.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Science-fiction drama centered on language, time perception, grief, love, and whether knowing the future changes how life should be lived.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Episode discussion focused less on act structure and more on fate, randomness, love, and accepting life with knowledge of pain.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; If you could press a button and see the rest of your life, would you want to know?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Choose love over fear; the ending is about accepting joy even knowing grief is coming.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The filler episodes of life are what make life feel alive.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Fate&lt;/li&gt;
+      &lt;li&gt;language&lt;/li&gt;
+      &lt;li&gt;love&lt;/li&gt;
+      &lt;li&gt;grief&lt;/li&gt;
+      &lt;li&gt;randomness&lt;/li&gt;
+      &lt;li&gt;choice&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+  &lt;p&gt;&lt;strong&gt;Archive Note:&lt;/strong&gt; A-tier philosophical episode.&lt;/p&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Style-driven getaway driver movie scored by music.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; What song did this movie remind you of?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The musical detail makes it theater-friendly.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; This is basically a two-hour music video.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Music&lt;/li&gt;
+      &lt;li&gt;crime&lt;/li&gt;
+      &lt;li&gt;technology aging&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;p&gt;Act 1: No Clipping Reality | Act 2: Endless Yellow | Act 3: Escape the Liminal&lt;/p&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;A man becomes trapped in the mysterious Backrooms, an endless maze of yellow hallways, while a strange scientific experiment and personal psychological struggles unfold around him.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;p&gt;Act 1 introduces the maze and confused premise. Act 2 follows prolonged wandering through the Backrooms while the hosts question the film’s purpose. Act 3 attempts to connect the maze to psychology and identity, but leaves most questions unanswered.&lt;/p&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Why did this movie become popular when the hosts found almost no story, character development, or payoff?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The film feels like a maze without a destination. Every time a theme appears, the movie abandons it before developing a meaningful journey.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The Backrooms works better as a short-form internet concept than a feature-length film. Stretching a YouTube idea into two hours exposed the lack of story.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Is the movie a deep metaphor about the human mind, or simply an incoherent story that audiences are overanalyzing?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Isolation&lt;/li&gt;
+      &lt;li&gt;loneliness&lt;/li&gt;
+      &lt;li&gt;mental health&lt;/li&gt;
+      &lt;li&gt;liminal spaces&lt;/li&gt;
+      &lt;li&gt;identity&lt;/li&gt;
+      &lt;li&gt;meaning-making&lt;/li&gt;
+      &lt;li&gt;storytelling versus concept&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;WOOM included chasing your dreams in 2026, Yung Miami/India Arie, Smartest Person in the Room, NBA Free Agency, Gold Medal Theory, and Top 3 TV episodes.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Cult comedy about Nisi and Mickey heading to Los Angeles, landing in a Beverly Hills mansion, and winning over a wealthy older man while chasing their business dream.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act I: From Georgia to Beverly Hills — diner, club, video audition, and the $10,000 scheme.&lt;/li&gt;
+    &lt;li&gt;Act II: The Makeover of a Mansion — Nisi and Mickey transform the mansion’s vibe.&lt;/li&gt;
+    &lt;li&gt;Act III: The Real Princesses — the scheme unravels and loyalty wins out.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; What hybrid business would we open with our podcast studio?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; This is basically Spendat: The Movie.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Raleigh needs an actual greasy-spoon breakfast diner, not brunch.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;90s comedy&lt;/li&gt;
+      &lt;li&gt;class&lt;/li&gt;
+      &lt;li&gt;fish-out-of-water&lt;/li&gt;
+      &lt;li&gt;friendship&lt;/li&gt;
+      &lt;li&gt;hood classics&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Wedding ensemble drama where Harper’s novel threatens friendships.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Does a secret like that ever truly stay buried?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Harper is the protagonist but also basically the villain.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Fiction inspired by true events needs plausible deniability.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Friendship&lt;/li&gt;
+      &lt;li&gt;loyalty&lt;/li&gt;
+      &lt;li&gt;betrayal&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Marcus Graham meets his match and reassesses ego, dating, and control.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Is this movie good?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Eddie Murphy is a strong dramatic actor among comedians.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Halle Berry as the everyday woman is ridiculous.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Dating&lt;/li&gt;
+      &lt;li&gt;ego&lt;/li&gt;
+      &lt;li&gt;image&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Hip-hop friendship romance about Dre and Sidney realizing the metaphor was love.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; When did you fall in love with hip-hop?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie is the article voiceover using hip-hop as a love metaphor.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Before rap became about getting a bag, there was more collaboration.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Hip-hop&lt;/li&gt;
+      &lt;li&gt;friendship&lt;/li&gt;
+      &lt;li&gt;love&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Dystopian escort story built around fertility collapse, government breakdown, and survival.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Do you have a go bag?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The future looking old shows social collapse creatively.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Post-apocalyptic movies are inherently conservative.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Collapse&lt;/li&gt;
+      &lt;li&gt;infrastructure&lt;/li&gt;
+      &lt;li&gt;survival&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: The Shadows Over Gotham | Act 2: The Escalation of Chaos | Act 3: The Soul of Gotham&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Batman, Jim Gordon, and Harvey Dent attempt to eliminate organized crime in Gotham while the Joker unleashes escalating chaos, forcing every major character to confront difficult moral choices.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: Joker’s bank heist establishes his intelligence, unpredictability, and agenda while Batman, Gordon, and Dent begin their alliance.&lt;/li&gt;
+    &lt;li&gt;Act 2: Joker’s attacks escalate as the hosts discuss Batman’s no-kill rule, Joker’s philosophy, and Nolan’s storytelling.&lt;/li&gt;
+    &lt;li&gt;Act 3: Harvey Dent becomes Two-Face, Batman accepts blame to preserve hope, and the hosts examine the film’s legacy.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was Gotham better off preserving Harvey Dent’s heroic image, even if it required lying to the public?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie transcends the genre because nearly every major character faces a difficult moral choice with real consequences.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The film succeeds because the good guys actually lose. Actions have consequences, victories are costly, and the stakes feel permanent.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Was Batman right to refuse to kill the Joker despite the destruction and lives lost?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Order vs. chaos&lt;/li&gt;
+      &lt;li&gt;burden of heroism&lt;/li&gt;
+      &lt;li&gt;moral compromise&lt;/li&gt;
+      &lt;li&gt;public faith and symbolism&lt;/li&gt;
+      &lt;li&gt;law versus vigilantism&lt;/li&gt;
+      &lt;li&gt;fragility of civilization&lt;/li&gt;
+      &lt;li&gt;sacrifice&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Neighborhood comedy about Craig, Smokey, Deebo, and one long Friday.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Is Pineapple Express the white Friday?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Pineapple Express is the white Friday.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Getting fired on your day off is egregious.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Neighborhood&lt;/li&gt;
+      &lt;li&gt;comedy&lt;/li&gt;
+      &lt;li&gt;friendship&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Game-night comedy where a murder mystery becomes a real kidnapping case.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; If you had a house in the suburbs, would you host?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Bring back cool credits in movies.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Jesse Plemons is the saving grace.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Hosting&lt;/li&gt;
+      &lt;li&gt;games&lt;/li&gt;
+      &lt;li&gt;suburbs&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Sixth-grade coming-of-age comedy about friendship and getting older.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Are you still cool with anyone from grade school?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie illustrates how stupid kids are.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The Black kid gets something to do beyond being Black.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Childhood&lt;/li&gt;
+      &lt;li&gt;friendship&lt;/li&gt;
+      &lt;li&gt;growing up&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Legal/family drama about a lawyer defending his estranged judge father.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was the bathroom scene the most powerful scene?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Opening relics show each family member’s role.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Robert Downey Jr. is elite; Marvel took serious roles from us.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Family&lt;/li&gt;
+      &lt;li&gt;fathers&lt;/li&gt;
+      &lt;li&gt;courtrooms&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Moral-dilemma courtroom premise; movie section in rundown was mostly blank.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; What does justice require when protecting yourself could condemn someone else?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Needs transcript pass.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Needs transcript pass.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Justice&lt;/li&gt;
+      &lt;li&gt;conscience&lt;/li&gt;
+      &lt;li&gt;self-preservation&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Sports romance about Monica and Quincy balancing love, family, and ambition.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was Monica wrong for leaving because of curfew?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie aged well and has strong family/feminist messaging.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; “Let’s play for your heart” is corny.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Love&lt;/li&gt;
+      &lt;li&gt;ambition&lt;/li&gt;
+      &lt;li&gt;family&lt;/li&gt;
+      &lt;li&gt;sports&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Romantic drama about poetry, timing, vulnerability, and whether love is real or just a thing.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was Darius who Nina wanted, or who was there when she was tired?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Nina loved how Darius made her feel more than she loved him.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Everyone is pretending to like jazz.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Romance&lt;/li&gt;
+      &lt;li&gt;art&lt;/li&gt;
+      &lt;li&gt;timing&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Family comedy revisited through an adult lens around divorce, parenting, and responsibility.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Did this movie age well?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Robin Williams at peak powers makes this a five-star classic.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; As an adult, Daniel looks like a man-child Miranda had to parent with.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Divorce&lt;/li&gt;
+      &lt;li&gt;parenting&lt;/li&gt;
+      &lt;li&gt;nostalgia&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Teen New York rom-com centered on music, technology, and one-night adventure.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; What five acts would you do anything to see live?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; After a breakup, delete everything or at least hide it.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The movie is a dated technology museum: iPod, burned CDs, flip phones.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Music&lt;/li&gt;
+      &lt;li&gt;NYC&lt;/li&gt;
+      &lt;li&gt;dating&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: The One Wish Willow | Act 2: Love Turned Unhinged | Act 3: The Price of Control&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; A shy record-store employee uses a supernatural charm to make childhood friend Nikki love him above everything else, turning unrequited longing into violent possession.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1 establishes Bear’s wish, Nikki’s lack of romantic interest, and Ian’s concealed history with her. Act 2 tracks the wish escalating through isolation, control, and violence. Act 3 confronts Bear’s responsibility, Nikki’s attempts to resist, and the deadly consequences of forced devotion.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Does unrequited love count as real love if it is never returned?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Nikki’s performance remains magnetic while small visual details suggest the real Nikki is fighting the wish throughout the movie.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Bear’s longing is relatable, but getting exactly what he wished for exposes the danger of confusing control with love.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Is Bear the villain, an immature young man trapped by an impulsive wish, or both?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Be careful what you wish for&lt;/li&gt;
+      &lt;li&gt;agency and coercion&lt;/li&gt;
+      &lt;li&gt;unrequited love&lt;/li&gt;
+      &lt;li&gt;attachment&lt;/li&gt;
+      &lt;li&gt;youthful insecurity&lt;/li&gt;
+      &lt;li&gt;control versus genuine affection&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Christopher Nolan epic about Odysseus returning home after the Trojan War.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Is this Matt Damon’s best role?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The Calypso “let go” idea works: surrender is not giving up.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The Cyclops sequence is the ultimate rewatch scene and proves what practical effects can do.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Journey&lt;/li&gt;
+      &lt;li&gt;mythology&lt;/li&gt;
+      &lt;li&gt;war&lt;/li&gt;
+      &lt;li&gt;homecoming&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: The Rivalry Begins | Act 2: The Illusion of Sacrifice | Act 3: The Ultimate Trick&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Two rival magicians in Victorian London become consumed by obsession after a fatal stage accident, sacrificing relationships, identities, and lives to create the ultimate illusion.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: A tragic water-tank accident divides the magicians and begins a destructive cycle of rivalry and sabotage.&lt;/li&gt;
+    &lt;li&gt;Act 2: A teleportation illusion intensifies the feud, leading Angier toward Tesla while Borden’s devotion to craft strains every relationship.&lt;/li&gt;
+    &lt;li&gt;Act 3: The secrets behind both illusions are revealed, exposing the human cost of obsession, sacrifice, and living a double life.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Did Borden tie the wrong knot, and did Borden truly know which knot was tied?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The screenplay’s symbolism, paired birds, foreshadowing, blocking, and mirrored rivalries make every scene necessary and reward immediate rewatching.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The twist holds up because the movie stays faithful to its clues; the twin performance, missing fingers, and divided relationships all remain consistent.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Is Angier the villain, or is Angier’s escalating cruelty understandable after watching a spouse die during Borden’s trick?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Obsession&lt;/li&gt;
+      &lt;li&gt;sacrifice&lt;/li&gt;
+      &lt;li&gt;rivalry&lt;/li&gt;
+      &lt;li&gt;identity&lt;/li&gt;
+      &lt;li&gt;showmanship versus craft&lt;/li&gt;
+      &lt;li&gt;passion&lt;/li&gt;
+      &lt;li&gt;deception&lt;/li&gt;
+      &lt;li&gt;divided lives&lt;/li&gt;
+      &lt;li&gt;the cost of applause&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: A Job Before the Fall&lt;/li&gt;
+    &lt;li&gt;Act 2: Paranoia in the Warehouse&lt;/li&gt;
+    &lt;li&gt;Act 3: Trust Runs Out&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt;&lt;/p&gt;
+  &lt;p&gt;After a diamond heist collapses into chaos, a crew of criminals regroups in a warehouse and begins searching for the rat among them. As suspicion grows, relationships fracture and the aftermath becomes more important than the robbery itself.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: Discussion of the crew&amp;#39;s structure, robbery planning, trust, conspiracy theories, and Tarantino&amp;#39;s early career.&lt;/li&gt;
+    &lt;li&gt;Act 2: Analysis of Mr. Blonde, the undercover storyline, the famous tipping scene, and the film&amp;#39;s cultural reputation.&lt;/li&gt;
+    &lt;li&gt;Act 3: Debate over whether the movie is genuinely great or simply pretentious, plus discussion of alternative endings and Tarantino&amp;#39;s evolution as a filmmaker.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Is Reservoir Dogs actually a great movie, or has its reputation been elevated because Tarantino later became one of the most acclaimed directors of all time?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie feels more culturally important than it feels enjoyable today. Its influence on later filmmakers is undeniable, but many of its characters and story elements feel underdeveloped on rewatch.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Reservoir Dogs may be the victim of retrospective praise. People love Pulp Fiction so much that they project some of that greatness backward onto Tarantino&amp;#39;s debut feature.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Is it better to commit a robbery with close friends or complete strangers, and does Reservoir Dogs prove that both approaches are doomed to fail?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Trust vs. self-preservation&lt;/li&gt;
+      &lt;li&gt;Loyalty and betrayal&lt;/li&gt;
+      &lt;li&gt;The psychology of lying&lt;/li&gt;
+      &lt;li&gt;Reputation versus reality&lt;/li&gt;
+      &lt;li&gt;Criminal organizations&lt;/li&gt;
+      &lt;li&gt;Group dynamics under pressure&lt;/li&gt;
+      &lt;li&gt;The costs of paranoia&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Coming-of-age baseball classic about childhood, summer, and neighborhood friendship.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Are you still friends with anyone from your childhood neighborhood?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Heroes get remembered and legends never die.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Adults should get one summer off every decade.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Childhood&lt;/li&gt;
+      &lt;li&gt;friendship&lt;/li&gt;
+      &lt;li&gt;nostalgia&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Gothic mystery/horror built on supernatural skepticism and Tim Burton atmosphere.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Would you rather be the writer or director?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Johnny Depp and Tim Burton are an underrated actor-director collaboration.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The B-plot is usually the vegetables you sneak into the story.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Mystery&lt;/li&gt;
+      &lt;li&gt;supernatural&lt;/li&gt;
+      &lt;li&gt;worldbuilding&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Roc-A-Fella cult crime movie about ABM taking over North Philly.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was this the OG Tubi movie?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; This is five-star classic Black cinema, warts and all.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; If you remove the good parts of Goodfellas, what remains is State Property.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Nostalgia&lt;/li&gt;
+      &lt;li&gt;crime&lt;/li&gt;
+      &lt;li&gt;rap culture&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Drama about early-onset Alzheimer’s, identity, memory, and family care.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Would you use genetic testing to edit chronic illness out?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The “most disappointing” child saw Alice the clearest.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Alice likely masked the disease longer because intelligence let her compensate.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Memory&lt;/li&gt;
+      &lt;li&gt;identity&lt;/li&gt;
+      &lt;li&gt;illness&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Original fantasy/drama about a man hearing the narrator of his life.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; If a voice narrated your life, what genre would it be?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Autopilot can make you feel like a side character in your own life.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Shout out to original movies.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Routine&lt;/li&gt;
+      &lt;li&gt;mortality&lt;/li&gt;
+      &lt;li&gt;originality&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; 80s party comedy about career pressure, lying, and adulthood.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; What was your favorite Grand Theft Auto?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; It is fun practice to extract conversation from a mediocre movie.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; White Friday minus compelling characters and being funny.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Adulthood&lt;/li&gt;
+      &lt;li&gt;nostalgia&lt;/li&gt;
+      &lt;li&gt;pressure&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;p&gt;Act 1: The Perfect Week Begins | Act 2: Truth Enters The Room | Act 3: Wedding Day Reckoning&lt;/p&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;Days before their wedding, Emma and Charlie’s seemingly perfect relationship is shattered by a shocking confession from Emma’s past, forcing everyone around them to confront trust, forgiveness, and identity.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;p&gt;Act 1 establishes their romance and wedding preparations. Act 2 detonates the story with Emma’s revelation that she once planned a school shooting. Act 3 follows the emotional fallout, wedding chaos, and ambiguous reconciliation.&lt;/p&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Is Emma’s revelation alone enough to call off the wedding, or is the larger issue everything else surrounding her character?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The film feels like a 100-minute panic attack, using anxiety, awkwardness, and emotional tension to place viewers directly in Charlie’s perspective.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The biggest red flag was not the confession itself, but Emma reaching adulthood with virtually no close friendships or meaningful relationships.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Do Emma and Charlie survive as a couple after the ending, or was the damage too large to overcome?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Forgiveness&lt;/li&gt;
+      &lt;li&gt;trust&lt;/li&gt;
+      &lt;li&gt;hidden identity&lt;/li&gt;
+      &lt;li&gt;mental health&lt;/li&gt;
+      &lt;li&gt;love versus judgment&lt;/li&gt;
+      &lt;li&gt;emotional immaturity&lt;/li&gt;
+      &lt;li&gt;second chances&lt;/li&gt;
+      &lt;li&gt;relationship pressure&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: The Photo That Opens The Door&lt;/li&gt;
+    &lt;li&gt;Act 2: Parallel Lives, Parallel Problems&lt;/li&gt;
+    &lt;li&gt;Act 3: Choosing What To Carry Forward&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt;&lt;/p&gt;
+  &lt;p&gt;After her mother&amp;#39;s death, Mae discovers a photograph and a series of unanswered questions about her family&amp;#39;s history. Her search for answers brings her together with journalist Michael Block, sparking a romance while two generations of love stories unfold in parallel.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act 1: The hosts discuss Issa Rae&amp;#39;s performance, the film&amp;#39;s premise, and the lack of chemistry between the leads.&lt;/li&gt;
+    &lt;li&gt;Act 2: Focus shifts to the dual timelines, comparisons to Love Jones, the soundtrack, and the film&amp;#39;s incomplete character arcs.&lt;/li&gt;
+    &lt;li&gt;Act 3: Discussion centers on letters, family secrets, inherited memories, and why the film never fully delivers on its emotional potential.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Should Michael have pursued a serious relationship with Mae while actively preparing to take a job in another country?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie contains the ingredients for a meaningful story about Black motherhood, ambition, generational wounds, and family legacy, but never fully commits to developing any of those ideas.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; The film feels like two separate movies stitched together. The flashbacks and present-day romance rarely connect in a meaningful way, leaving both storylines underdeveloped.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; Was this a genuine romance, or was it simply a less compelling attempt to recreate the magic of Love Jones for a newer generation?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Family legacy&lt;/li&gt;
+      &lt;li&gt;Motherhood&lt;/li&gt;
+      &lt;li&gt;Generational trauma&lt;/li&gt;
+      &lt;li&gt;Ambition versus relationships&lt;/li&gt;
+      &lt;li&gt;Memory and grief&lt;/li&gt;
+      &lt;li&gt;Love across generations&lt;/li&gt;
+      &lt;li&gt;Identity and self-discovery&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Holiday family drama about secrets, siblings, debt, relationships, and reunion.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Does your family do a big Christmas?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Black parent logic: you cannot sing, but you can ride a motorcycle.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Christmas family movies all have the same plot, but it works.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Family&lt;/li&gt;
+      &lt;li&gt;holidays&lt;/li&gt;
+      &lt;li&gt;secrets&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Horror mystery about a town after almost an entire class disappears.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Why did no one have guns?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Camera work and child narration build confusion and suspense.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Act one and two are great; the ending falls apart.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Grief&lt;/li&gt;
+      &lt;li&gt;suspense&lt;/li&gt;
+      &lt;li&gt;endings&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Sports comedy about hustling, partnership, money, and relationships in 90s LA.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Was Gloria right to leave?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; Gloria was right to leave because of repeated money-management issues.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Why don’t these people just get jobs?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Money&lt;/li&gt;
+      &lt;li&gt;relationships&lt;/li&gt;
+      &lt;li&gt;basketball&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Run down and/or transcript notes preserved in original archive; this page keeps the same original-section layout for OneNote import.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Summary:&lt;/strong&gt; Home-invasion slasher discussed as dumb, fun, and Halloween-curve entertainment.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Act / Segment Breakdown: use original rundown act notes in OneNote as needed; this import preserves the BEFORE/AFTER page structure.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Why is everyone doing a contract killing the hard way?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; This movie only works if everyone is stupid.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; I love a good stupid slasher; grading it on a Halloween curve.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Horror logic&lt;/li&gt;
+      &lt;li&gt;survival&lt;/li&gt;
+      &lt;li&gt;Halloween&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
 </sst>
 </file>
 
@@ -6081,12 +6922,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -6114,6 +6949,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -6140,32 +6980,22 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -6173,6 +7003,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6513,863 +7346,751 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14" style="12" customWidth="1"/>
-    <col min="5" max="5" width="72" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="72" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" style="8" customWidth="1"/>
+    <col min="5" max="5" width="72" customWidth="1"/>
+    <col min="6" max="6" width="53.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>145</v>
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>147</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>1957</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2" s="7">
         <v>5</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="7">
         <v>5</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="6" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="364.5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="B3" s="4">
+        <v>1999</v>
+      </c>
+      <c r="C3" s="7">
+        <v>3.5</v>
+      </c>
+      <c r="D3" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="4">
+        <v>2016</v>
+      </c>
+      <c r="C4" s="8">
+        <v>5</v>
+      </c>
+      <c r="D4" s="8">
+        <v>4</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:6" ht="378" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B5" s="4">
+        <v>2017</v>
+      </c>
+      <c r="C5" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D5" s="8">
+        <v>3</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0</v>
+      </c>
+      <c r="D6" s="8">
+        <v>1</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1997</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="E7" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
         <v>1999</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C8" s="8">
+        <v>4</v>
+      </c>
+      <c r="D8" s="8">
+        <v>4</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1992</v>
+      </c>
+      <c r="C9" s="8">
+        <v>3</v>
+      </c>
+      <c r="D9" s="8">
+        <v>2</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>2002</v>
+      </c>
+      <c r="C10" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="D10" s="8">
+        <v>4</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4">
+        <v>2006</v>
+      </c>
+      <c r="C11" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="8">
+        <v>3</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>2008</v>
+      </c>
+      <c r="C12" s="8">
+        <v>5</v>
+      </c>
+      <c r="D12" s="8">
+        <v>5</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="F12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="391.5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4">
+        <v>1995</v>
+      </c>
+      <c r="C13" s="8">
         <v>3.5</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D13" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="405" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4">
+        <v>2018</v>
+      </c>
+      <c r="C14" s="8">
+        <v>2</v>
+      </c>
+      <c r="D14" s="8">
+        <v>2</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4">
+        <v>2019</v>
+      </c>
+      <c r="C15" s="8">
+        <v>3</v>
+      </c>
+      <c r="D15" s="8">
+        <v>3</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>2014</v>
+      </c>
+      <c r="C16" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D16" s="8">
+        <v>3</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="405" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>2024</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="E17" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>2000</v>
+      </c>
+      <c r="C18" s="8">
+        <v>5</v>
+      </c>
+      <c r="D18" s="8">
+        <v>3</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="F18" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4">
+        <v>1997</v>
+      </c>
+      <c r="C19" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D19" s="8">
+        <v>4</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1993</v>
+      </c>
+      <c r="C20" s="8">
+        <v>5</v>
+      </c>
+      <c r="D20" s="8">
+        <v>5</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4">
+        <v>2008</v>
+      </c>
+      <c r="C21" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D21" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="F21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C22" s="8">
+        <v>4</v>
+      </c>
+      <c r="D22" s="8">
+        <v>4</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C23" s="8">
+        <v>5</v>
+      </c>
+      <c r="D23" s="8">
+        <v>5</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4">
+        <v>2006</v>
+      </c>
+      <c r="C24" s="8">
+        <v>5</v>
+      </c>
+      <c r="D24" s="8">
+        <v>5</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4">
+        <v>1992</v>
+      </c>
+      <c r="C25" s="8">
         <v>2.5</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="G3" t="s">
-        <v>109</v>
+      <c r="D25" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F25" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="26" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1993</v>
+      </c>
+      <c r="C26" s="8">
         <v>5</v>
       </c>
-      <c r="B4" s="5">
-        <v>2016</v>
-      </c>
-      <c r="C4" s="12">
+      <c r="D26" s="8">
         <v>5</v>
       </c>
-      <c r="D4" s="12">
+      <c r="E26" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4">
+        <v>1999</v>
+      </c>
+      <c r="C27" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D27" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4">
+        <v>2002</v>
+      </c>
+      <c r="C28" s="8">
+        <v>5</v>
+      </c>
+      <c r="D28" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4">
+        <v>2014</v>
+      </c>
+      <c r="C29" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="D29" s="8">
+        <v>5</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4">
+        <v>2006</v>
+      </c>
+      <c r="C30" s="8">
+        <v>3</v>
+      </c>
+      <c r="D30" s="8">
+        <v>2</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F30" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4">
+        <v>2011</v>
+      </c>
+      <c r="C31" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D31" s="8">
+        <v>1</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4">
+        <v>2026</v>
+      </c>
+      <c r="C32" s="8">
         <v>4</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" t="s">
-        <v>110</v>
+      <c r="D32" s="8">
+        <v>4</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="F32" t="s">
+        <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5">
-        <v>2017</v>
-      </c>
-      <c r="C5" s="12">
+    <row r="33" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4">
+        <v>2020</v>
+      </c>
+      <c r="C33" s="8">
+        <v>2</v>
+      </c>
+      <c r="D33" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4">
+        <v>2007</v>
+      </c>
+      <c r="C34" s="8">
+        <v>3</v>
+      </c>
+      <c r="D34" s="8">
         <v>3.5</v>
       </c>
-      <c r="D5" s="12">
+      <c r="E34" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="F34" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4">
+        <v>2025</v>
+      </c>
+      <c r="C35" s="8">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>111</v>
+      <c r="D35" s="8">
+        <v>3</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F35" t="s">
+        <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="5">
-        <v>2026</v>
-      </c>
-      <c r="C6" s="12">
-        <v>0</v>
-      </c>
-      <c r="D6" s="12">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>112</v>
+    <row r="36" spans="1:6" ht="405" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4">
+        <v>1992</v>
+      </c>
+      <c r="C36" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="D36" s="8">
+        <v>4</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="F36" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="5">
-        <v>1997</v>
-      </c>
-      <c r="C7" s="12"/>
-      <c r="E7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="5">
-        <v>1999</v>
-      </c>
-      <c r="C8" s="12">
+    <row r="37" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>2011</v>
+      </c>
+      <c r="C37" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="D37" s="8">
         <v>4</v>
       </c>
-      <c r="D8" s="12">
-        <v>4</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5">
-        <v>1992</v>
-      </c>
-      <c r="C9" s="12">
-        <v>3</v>
-      </c>
-      <c r="D9" s="12">
-        <v>2</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5">
-        <v>2002</v>
-      </c>
-      <c r="C10" s="12">
-        <v>4.5</v>
-      </c>
-      <c r="D10" s="12">
-        <v>4</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="5">
-        <v>2006</v>
-      </c>
-      <c r="C11" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D11" s="12">
-        <v>3</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="5">
-        <v>2008</v>
-      </c>
-      <c r="C12" s="12">
-        <v>5</v>
-      </c>
-      <c r="D12" s="12">
-        <v>5</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="5">
-        <v>1995</v>
-      </c>
-      <c r="C13" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D13" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="5">
-        <v>2018</v>
-      </c>
-      <c r="C14" s="12">
-        <v>2</v>
-      </c>
-      <c r="D14" s="12">
-        <v>2</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="5">
-        <v>2019</v>
-      </c>
-      <c r="C15" s="12">
-        <v>3</v>
-      </c>
-      <c r="D15" s="12">
-        <v>3</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G15" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="5">
-        <v>2014</v>
-      </c>
-      <c r="C16" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D16" s="12">
-        <v>3</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="5">
-        <v>2024</v>
-      </c>
-      <c r="C17" s="12"/>
-      <c r="E17" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="5">
-        <v>2000</v>
-      </c>
-      <c r="C18" s="12">
-        <v>5</v>
-      </c>
-      <c r="D18" s="12">
-        <v>3</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="5">
-        <v>1997</v>
-      </c>
-      <c r="C19" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D19" s="12">
-        <v>4</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G19" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="5">
-        <v>1993</v>
-      </c>
-      <c r="C20" s="12">
-        <v>5</v>
-      </c>
-      <c r="D20" s="12">
-        <v>5</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G20" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B21" s="5">
-        <v>2008</v>
-      </c>
-      <c r="C21" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D21" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G21" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="5">
-        <v>2026</v>
-      </c>
-      <c r="C22" s="12">
-        <v>4</v>
-      </c>
-      <c r="D22" s="12">
-        <v>4</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G22" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" s="5">
-        <v>2026</v>
-      </c>
-      <c r="C23" s="12">
-        <v>5</v>
-      </c>
-      <c r="D23" s="12">
-        <v>5</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>65</v>
-      </c>
-      <c r="B24" s="5">
-        <v>2006</v>
-      </c>
-      <c r="C24" s="12">
-        <v>5</v>
-      </c>
-      <c r="D24" s="12">
-        <v>5</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G24" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="E37" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="F37" t="s">
         <v>68</v>
-      </c>
-      <c r="B25" s="5">
-        <v>1992</v>
-      </c>
-      <c r="C25" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D25" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G25" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>71</v>
-      </c>
-      <c r="B26" s="5">
-        <v>1993</v>
-      </c>
-      <c r="C26" s="12">
-        <v>5</v>
-      </c>
-      <c r="D26" s="12">
-        <v>5</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G26" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>74</v>
-      </c>
-      <c r="B27" s="5">
-        <v>1999</v>
-      </c>
-      <c r="C27" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D27" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G27" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>77</v>
-      </c>
-      <c r="B28" s="5">
-        <v>2002</v>
-      </c>
-      <c r="C28" s="12">
-        <v>5</v>
-      </c>
-      <c r="D28" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G28" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="5">
-        <v>2014</v>
-      </c>
-      <c r="C29" s="12">
-        <v>4.5</v>
-      </c>
-      <c r="D29" s="12">
-        <v>5</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="G29" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>83</v>
-      </c>
-      <c r="B30" s="5">
-        <v>2006</v>
-      </c>
-      <c r="C30" s="12">
-        <v>3</v>
-      </c>
-      <c r="D30" s="12">
-        <v>2</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="G30" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>86</v>
-      </c>
-      <c r="B31" s="5">
-        <v>2011</v>
-      </c>
-      <c r="C31" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D31" s="12">
-        <v>1</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G31" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B32" s="5">
-        <v>2026</v>
-      </c>
-      <c r="C32" s="12">
-        <v>4</v>
-      </c>
-      <c r="D32" s="12">
-        <v>4</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G32" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>92</v>
-      </c>
-      <c r="B33" s="5">
-        <v>2020</v>
-      </c>
-      <c r="C33" s="12">
-        <v>2</v>
-      </c>
-      <c r="D33" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="G33" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>95</v>
-      </c>
-      <c r="B34" s="5">
-        <v>2007</v>
-      </c>
-      <c r="C34" s="12">
-        <v>3</v>
-      </c>
-      <c r="D34" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="G34" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>98</v>
-      </c>
-      <c r="B35" s="5">
-        <v>2025</v>
-      </c>
-      <c r="C35" s="12">
-        <v>3</v>
-      </c>
-      <c r="D35" s="12">
-        <v>3</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="G35" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>101</v>
-      </c>
-      <c r="B36" s="5">
-        <v>1992</v>
-      </c>
-      <c r="C36" s="12">
-        <v>3.5</v>
-      </c>
-      <c r="D36" s="12">
-        <v>4</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="G36" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="5">
-        <v>2011</v>
-      </c>
-      <c r="C37" s="12">
-        <v>2.5</v>
-      </c>
-      <c r="D37" s="12">
-        <v>4</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="G37" t="s">
-        <v>140</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{8E5B87CC-F717-4172-93E2-C446A611ADD5}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{8E5B87CC-F717-4172-93E2-C446A611ADD5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -7386,11 +8107,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>141</v>
+      <c r="A1" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>148</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
@@ -7398,284 +8119,284 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>149</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>150</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>151</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>152</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>153</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>154</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>155</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>157</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>158</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>159</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>160</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>161</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>162</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>163</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>164</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>165</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>166</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>167</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>168</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>169</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>170</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>171</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>172</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>173</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>174</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>175</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>176</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>177</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>178</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>179</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>180</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>181</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>182</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>104</v>
+        <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>183</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix mobile menu button styling and deploy updated WOOM and Movie archives
</commit_message>
<xml_diff>
--- a/Movie Archive Inputs.xlsx
+++ b/Movie Archive Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A11AB435-A7A4-42DF-BD98-EE62D6A119C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD4D2A1-218C-4982-BCEA-37AB0A8980C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movie Ratings" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="150">
   <si>
     <t>12 Angry Men</t>
   </si>
@@ -6909,6 +6909,190 @@
     &lt;/ul&gt;
   &lt;/div&gt;
 &lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>Hustlers</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Episode Rundown&lt;/h3&gt;
+  &lt;h3&gt;Front Half / Episode Segments&lt;/h3&gt;
+  &lt;p&gt;Act 1: The Education | Act 2: The Recession Pivot | Act 3: The Cost of the Game&lt;/p&gt;
+  &lt;h3&gt;Movie / Episode Basics&lt;/h3&gt;
+  &lt;p&gt;A young stripper learns the business from Ramona before the 2008 financial crisis forces a group of dancers into an increasingly dangerous criminal scheme targeting wealthy clients.&lt;/p&gt;
+  &lt;h3&gt;Act / Segment Breakdown&lt;/h3&gt;
+  &lt;p&gt;Act 1 covers mentorship, strip-club culture, and power dynamics. Act 2 explores the economic fallout of 2008 and the women’s scam operation. Act 3 focuses on accountability, loyalty, criminal consequences, and moral ambiguity.&lt;/p&gt;
+  &lt;h3&gt;Episode Highlights&lt;/h3&gt;
+  &lt;p&gt;&lt;strong&gt;Best Question:&lt;/strong&gt; Did the women genuinely believe they were helping themselves survive, or were they simply rationalizing serious crimes?&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Jordan Insight:&lt;/strong&gt; The movie succeeds because everyone is morally compromised. The women, the customers, and the clubs all operate in shades of gray rather than simple heroes and villains.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Darius Insight:&lt;/strong&gt; Hustlers is one of the better films about the 2008 financial crisis because it captures how quickly economic desperation can push ordinary people toward extreme choices.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Best Debate:&lt;/strong&gt; If the genders were reversed, would audiences have celebrated the story the same way?&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Economic survival&lt;/li&gt;
+      &lt;li&gt;exploitation&lt;/li&gt;
+      &lt;li&gt;mentorship&lt;/li&gt;
+      &lt;li&gt;loyalty&lt;/li&gt;
+      &lt;li&gt;financial desperation&lt;/li&gt;
+      &lt;li&gt;gender dynamics&lt;/li&gt;
+      &lt;li&gt;accountability&lt;/li&gt;
+      &lt;li&gt;crime and rationalization&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>Jordan: Welcome to the Out the Trunk pod with Jordan and Darius. My name is Jordan. That's Jordan to be writing on all socials.
+Darius: And I'm Darius. That's these all up in area on all socials. And today we're.
+Jordan: Going to be talking about the movie Hustlers, what worked, what didn't, and whether the movie's big swings paid off. Let's get into it.
+Darius: Act 1, the education. Destiny enters a high pressure club world, learns from Ramona's confidence and strategy, and begins to understand the power dynamics behind performance, money, and survival. Off the rip, I feel like I'm an alien from a different planet because I do not enjoy strip clubs at all. And I get that that makes me alien to most men. But every time I go, I'm like, I just would rather be somewhere else right now. Like, I don't enjoy this. You know, I understand that makes me weird, but they're not for me. So a little fun fact about Darius.
+Jordan: Yeah, I've been a few times. It's cool. It's not my, not really my like regular type thing. We do know people who it is the regular thing. Yeah, I mean, it's all right. It's, you know, it's cool when you're with friends and they want to go. It's better to go with like your women friends. It's more enjoyable for everyone. From what I hear.
+Darius: I remember one of my favorite tweets was the guy who was like, dudes going to strip clubs. It's got to be so odd. It's like, hey, you guys want to go get some ****** together? Sure. What else we do it like? and I felt so seen because I was like, I thought I was the only one who thought that I'm just not into this.
+Jordan: No, it actually is nuts. It's like, because at no point in life would you be like, hey, you want to sit with me while I can dry up?
+Darius: Yeah, it's just, I'm not sure why this isn't as taboo. I mean, it's not taboo at all as ****. In some cities, it's like a restaurant with strippers in it.
+Jordan: I'm about to say, yeah, Atlanta and like New Orleans.
+Darius: Not for me. I've been to strip clubs all over the country. Mostly not at my idea. You know, bachelor parties, fellas want to go. I'm not a party hooper.
+Jordan: Yeah.
+Darius: So like, if the group's going, I'm not going to be like, this is a moral outbreak, you know, I just whatever. But yeah, yeah.
+Jordan: You know, Vegas Friendsgivings, Atlanta, you know, the whole thing.
+Darius: Oh, yeah. Y'all did DoorDash strippers after Thanksgiving dinner. I forgot about that. That was one of our best episodes.
+Jordan: It really was. I didn't. I didn't order them. I was just there. And while they were arrived at the location for the listeners.
+Darius: You know, it doesn't. It doesn't matter. You were there when the strippers were called up on the app. Yeah, that's and dropped off via in somebody's Honda Sonata. And yeah, the rest was history.
+Jordan: The rest is history. And in. My first note is JLo is fine as ****. That is a central plot point. That is a central plot point of the movie, literally, because she is a stripper. Also, she's an amazing actress. And I know we like to she's fun to like make fun of on social media and stuff like that. But she's really super talented. And I'd love to see her more movies and especially like more villain roles because she was phenomenal in this movie.
+Darius: Yeah, you she does. The IMDB is bloated because she does a lot of Netflix. Blop the slop.
+Jordan: Yeah.
+Darius: Like, you know, oh, someone kidnapped my kid. I'm going to go, you know, like she has a lot of slop on the Netflix and the.
+Jordan: Yeah, she does.
+Darius: But when she locks in and they give her a good script, she's up there.
+Jordan: You know, it's not too many that can **** with her.
+Darius: No, it's. Yeah. Yeah. Well, that's English. What else you got for act one?
+Jordan: I like how they broke down. like the psychology of the guys, like the profiles of what they look for when they're looking for a mark. They're like, look at his shoes, look at his watch, look at the permanent things, not the suits, because you can wear a nice suit for one day. That doesn't give away your lifestyle. Like how they broke down like, oh, this is the low level guy on Wall Street. This is the hedge fund exec. This is the whatever the term is. I don't know. I'm not bigging this to Wall Street. I mean, stocks, but the mid-level guys. I thought that was really cool how they kind of broke that down and showed the profiles. Also, it was insane even showing like their houses, like they all had crazy cribs, but there was still a vast difference in their classes.
+Darius: Yeah, it's like, especially when it comes to formal wear, the suits are dead. I mean, the shoes are a dead giveaway because everybody got two or three nice suits and you got to wear shoes every day. And so if your money is funny, you're not replenishing them. And they get beat or they're cheap to begin with. And it's just right. Yeah. The shoes are always you see a lot of, you know, nice to very nice suits and the shoes are busted and it's like, okay, you bought that one suit, you take care. And there's no shade. I own two suits. So granted, I don't really I don't wear that only use for them, but it's not like I have a closet full of suits either. And I have one pair of black dress shoes and one pair of brown dress shoes, and they're cheap. So I speak from experience.
+Jordan: So you know the mark in the club.
+Darius: No, no, I would never fall for any of these tricks.
+Jordan: I think, you know, that too.
+Darius: It's a lot. The the male ego is crazy because you see you get this a lot like dudes will touch down in Vegas and get drugged and robbed. And the story will be like, I walked in the club and these two women were interested in me and they asked me back to their room. And I'm like, have you ever had that kind of motion in your life?
+Jordan: Like outside of the movies, In Little.
+Darius: Rock, Arkansas, you've never had that kind of motion, but you touched down in Las Vegas and now you just can't keep them on for you.
+Jordan: Right.
+Darius: It never occurred to you that this is odd.
+Jordan: Yeah, and it's like, I mean, granted, it's different in the movies versus real life, but like in the movie, they weren't really hammered by the time girls got to them. So it really doesn't make any sense why you would fall for that.
+Darius: I've had it. I've just tried on me in Vegas. It's real. It's not like it happens just like that. Like you'll be sitting at a bar having your drink and a woman that two, like one woman, sometimes two that are just, it's just way too good to be true. Will come up to you and be like, Oh, when did you fly in? What do you do for a living? You're so funny. And they're just laughing at everything you say. And you're just like, I'm not that smooth.
+Jordan: Yeah, no. And I can't. And I don't want to afford you, even if I could.
+Darius: So there's like, you're a solid nine. I've never had one nine come up to me and be this friendly. Now, two in Vegas, like, come on, right?
+Jordan: Yeah.
+Darius: If it happens just like that, it was not a realistic.
+Jordan: Yeah, that's the crazy part to me. It's like, I don't know how they don't know. Like, it's like so obvious.
+Darius: And any time you see a picture of a dude after the fact, you like my guy.
+Jordan: Yeah, it's like when the cops read the articles and they were like, what a ****.
+Darius: It's like, dude, you know, fellas, be cognizant of the kind of emotion you have in your day-to-day. And then when you go to these cities, LA, Miami, Vegas, I have to say crazy nights can't happen because I've definitely, while traveling, the stars aligned and it was a good time. But you know, keep your wits about you. Don't get too overly drunk. If it's too good to be true.
+Jordan: It is.
+Darius: It probably is, man. You got to know.
+Jordan: You got to know.
+Darius: Now it's entirely possible.
+Jordan: Know what you look like?
+Darius: It's entirely possible to be out, you and the fellas at a club in Vegas and run into a bachelorette party. And they're good looking, but regular good looking.
+Jordan: Yeah, that makes sense.
+Darius: And you know, one of the bridesmaids is just in a great vacation mood. That's fine. But like a solid nine and her girlfriend come up is like, hey, you want to go have a threesome? It's like, you're going to wake.
+Jordan: Up with all your **** gone and you're not going to remember the last week of your life.
+Darius: At least put your wallet in the safe so you can get yourself something to eat the next day. They will take your socks if it's available.
+Jordan: And then you got to explain that to your bank and your wife or girlfriend, whoever you have, it's just, and then you, and then they're like, really, that's what happened to you? Like, and you didn't see that coming.
+Darius: It's just, it's not to say good nights can't happen on the road, because it does, especially in party cities where you're not the only person on vacation. You want to resort in Cancun, everyone's there's everyone there is Ain't got to worry about work, ain't got to worry about their kids, ain't got to worry about whatever. A good time, hair down. But just be aware of where you rank, what kind of emotion you normally have, and weigh that against your current circumstances and ask yourself, does this make sense? You know.
+Jordan: Yeah. In the words of Boss Mandilo, it's a motion party. You cannot get in.
+Darius: Exactly, Ben. It's just, you know. But it does happen exactly like the movies. So let me ask you this. So they set up almost like a mentorship program between, I'm really bad at character names, but J-Lo's character and Constant Wu's character. And in a cutthroat business, like a strip club, where the money is finite, like you're working for, the money is not pooled, you know, can mentorship really exist in a business that's cutthroat where everyone's working for the same $100 that's available by the men on the floor.
+Jordan: Yeah, I don't. I'm sure I'm sure it happens. Like, I know it happens. But from an institutional standpoint, I don't believe so. Like, you know, you think about it. And also, Jayla's character is an older character in the like she's older, like the older lady in the strip club is not trying to help the young new girl. And like, that's just not plausible. Like, this is how they pay the bills, you know what I'm saying?
+Darius: Like, that's just literally age out. So.
+Jordan: Yeah, like, like Brett Ford wasn't trying to help Aaron Rodgers for a reason. You know what I'm saying?
+Darius: Like, I was actually going to bring up that example is like human beings are naturally cooperative because you'll see you'll see videos of Miles Garrett and Will Anderson and a couple of people working out and like. Miles Garrett has. Why would he help Will Anderson get better? Right. But that's just how people are, even though they're competing for the same trophy. It's just. We're just naturally a cooperative species. So I think even though it makes no actual sense, it's possible you see it happen. And that was my example of it happening was like sports where people, competitors in the off season will work out together and make each other better, which doesn't actually make any sense beyond our natural ability to cooperate and, you know, pool our resources. So.
+Jordan: Yeah, that's a good point. Yeah, like I mean, trying to think like I remember Ironically, that was it at a strip club one night with when it was others when we all went, we're all there, whatever. And the one girl was done working. And then the next girl was about to come out to work. And she was like, oh, that's my best friend. Like, make sure to give her a good tip. Like, you know, so there is some camaraderie there. But I had a friend, a childhood friend who was a dancer. And she would tell me like some of the **** that went on between the girls and I can't go to this club because this girl's boyfriend doesn't like me and he runs the door and, **** like that. So there is a very competitive, element to that field.
+Darius: I have a friend of mine who used to bounce at a strip club, and he said he broke up fights at least every other night between the strippers.
+Jordan: Yeah, makes sense.
+Darius: He was like, most of my bouncing was. because now that was my client or I saw him last week or you owe me 10% of da da da da da because my stage time was cut or.
+Jordan: Just tipping out and all that stuff.
+Darius: Tipping to the DJ for more another song and just it can be ruthless. Yeah, because the men there they're not most of them aren't throwing all of their money and so you have to right you're fighting for someone else's discretionary income um correct of which you know it's a limited resource so yeah you got anything else for act one?
+Jordan: Um this movie is loaded I hadn't seen this movie play since it came out and I forgot how many just how many people were in this movie they had everybody in here.
+Darius: And honestly what did this release 2018?
+Jordan: I think so. Maybe 16?
+Darius: I mean, this is probably Lizzo before the fame, right?
+Jordan: I think like right before or at the peak, 2019.
+Darius: So we probably did.
+Jordan: So she was kind of popping back.
+Darius: Yeah, but like Cardi B just had that.
+Jordan: She had just popped.
+Darius: Yeah. It's a lot of people that this budget probably couldn't afford anymore. But it was it's cool. They all had little cameos and they all did. what they could with the time they had. And I enjoyed it, you know?
+Jordan: Me too. Me too. Did you have a favorite performance in the movie? Aside from J.Lo and constants, I guess I should say.
+Darius: The reporter, Kate Winslet, I think it was.
+Jordan: Julia Styles.
+Darius: Julia Styles Save the Last Dance. Yeah, I just thought I get to it later that I think that's kind of like a movie trope, but just the way she would react to the subject in the questioning, I thought if someone who listens to a lot of interview pods and watches a lot of journalism at work, I just thought she caught the nuances of that really, really well. There's an art to interviewing someone, when to interject, when to let them speak, when to, it's, you don't know what good interviewing is until you hear bad interviews.
+Jordan: See a bad interviewer?
+Darius: Like the super popular Joe Budden's pod, I think they are terrible interviewers. I never hear what the subject has to say. Yeah, they'll have a guest on and I'm like, can y'all let him answer the damn question? Why is he even here then? Like you just like, it's like. Right. And so she she got getting in and out of your cuts, asking the question and getting out of the way, not clearing your throat too much. I thought that she was really great as she did. She did a good job of acting like a great interviewer, so.
+Jordan: Yeah, that's true.
+Darius: Straving the last dance. What else you got for act one?
+Jordan: That's all I got for act one.
+Darius: Heading into act 2, the recession pivot, millennial shudder right there. Economic pressure changes the rules, forcing the women to reassess work, friendship, and risk as they look for stability in an unforgiving post-crash landscape. I have a particular affinity for movies about the financial crash, crash of 08 because that was when I entered the workforce for real. And, you know, for the kids, if you weren't around for that, it was it's impossible to explain to you how I knew people with like master degrees who were taking jobs at McDonald's because that was the job. That was all they could do. You know, it was it's it is Yeah, it was it was an era defining time. So where were you in a way? Were you still in school or what was going on in a way?
+Jordan: Yeah, I was in high school. I was a sophomore.
+Darius: All right, fair enough.
+Jordan: Yeah, I was. I luckily I was not. They didn't need me.
+Darius: Fair enough. Yeah, I it's. It's just, you know, it is a special place in my upbringing. So yeah, that's part of why I like this movie is because it captures the overnight change well like she comes back to the club and like it was empty it was empty and the things she had to do for the things she thought she'd never had to do for money like she has to do and you know obviously it's way different into the spectrum but like you know people with master's degrees never thought they'd have to apply at Wendy's and they had to because that's right he was and so yeah that kind of resonated with me in a way what you got for act two?
+Jordan: They did do a great job of showing what it's like trying to look for a job in a really ****** economy. And it's kind of interesting because I was thinking about this over the last few weeks and the conversation I had with my dad, maybe like close to a year ago. And I was trying to explain to him kind of what it's like now, you know, for like younger people. And I was like, I was like, we're the most educated underachievers of all time. like the job market, the way the job market is and competitiveness of it, the lack of, I won't say livable wages, but just, it's just really hard to get a comfortable job in a position that would really let you have the life that you want to have based on what we were told when we went to high school and went to college, and kind of the movie did a great job of showcasing that because, she did try to do the right thing she got an honest job you know she got a GED she was trying to go to school market went to hell and she can't even sell do retail and it's like I worked at a bar if I can that's talking to people all day like how can I not you know do retail and it's just like it feels like the days of like taking a shot on a candidate for like a job is kind of over and the job that scene did a great job of of showing that yeah that's what.
+Darius: People made the, I saw this point made on Twitter is like, what's with these jobs with these three, four, five rounds of interviews? And someone responded with, that's because they're all looking for a unicorn candidate instead of just like picking somebody and teaching them a job. And yeah, just like.
+Jordan: They don't want to train anymore.
+Darius: They don't want to train anymore. They want people who already know what they're already know the job. Not only that, but they just like, you know, I once had a mentor earlier in my career, he sat me down and he was like, one day you're going to have a team and on that team is going to be 10 people and you're going to have two to three superstar high productive employees. And you're going to have two to three. He's like, you're going to have two highly productive employees and you're going to have two pieces of ****. And you're going to have six people who just want to clock in, do their job and go home. Right. You nurture the people who want to be productive and get advanced and you help them nurture their career and you cycle out the pieces of **** to, you know, get them out of there. You leave the six people who just want to work and go home alone. Like, you know, like, and so it's almost like nobody wants employees that just want to work and go home. Everyone wants 10 superstars on a team and that's just not right. If it wasn't, if everyone was a superstar, I wouldn't be valuable. I always, that always resonated with me. And it's dated advice now because everyone wants 10 superstars, but he just was like, correct. Out of the 10 people, two are gonna be superstars, highly productive. You take care of them, you get them what they need. You help them develop their careers. So on and so forth. They get a little extra rope, so on and so forth. They get more privileges. But to cycle them out, leave the six that just wanna clock in, do their job, perform well. You know, get a meet expectations on their thing and go home with their families. And there's nothing wrong with that. And so we've lost that assets in work.
+Jordan: That's a great way to put it, because it feels like jobs view them as the pieces of ****. Like, you know, like I was talking about that with some friends of mine were telling me like they were looking for a job and they were saying like, let's say that their name was Jane Doe and they were like 5-2, for example. And they were saying like, I could look for a job for a girl named Jane and I wouldn't I wouldn't get it and it's like I could look for a job for a girl named Jane Doe and I wouldn't get a call back and it could be a job for a Jane Doe who's 5-2 and I still wouldn't get a call like you know what I mean and it's like because the ATS systems and the AI and the all the SEO and all that stuff it's more of a word problem than a resume you know what I'm saying it's It's more of an audition than an interview.
+Darius: It's funny because it's like you wouldn't ever actually want to do this because this is a free country. But I think a lot of industries would be better off with just auto sorting. Like this is we got 1000 college graduates this year. You get 10, you get 10, you know, like because and like almost like an NBA draft, but you know, that would never work. And you know, because there's a bunch of like civil rights issues that go with that.
+Jordan: And too many variables.
+Darius: But it's almost, it's the same as like the Netflix thing where if you have 1000 movies to watch, you're never going to pick one. If you're sitting there with 8 million applications, I want Jane Doe 52. Here's Jane Doe 51, she's out of here. Here's Doe Jane 56, she's out here. It's just like, you need to just make a decision. Stop waiting for the unicorn because unicorns by definition are exceedingly rare.
+Jordan: Correct.
+Darius: Yeah, I'm with you. It's it's.
+Jordan: And that unicorn would be over. But yeah, that's true. Yeah.
+Darius: And how long are you going to keep the unicorn, you know?
+Jordan: So that too. Yeah, it's very odd. And I feel like the the they run off good people because of the obsession with like metrics and the obsession with hyper productivity now, you know what I mean? It's like they'll, they'll say like, I don't want you to be a machine, but like actually work faster and harder and make less mistakes. Machines do that, you know what I mean?
+Darius: The, the, sorry, I lost my notes for, yeah, the, you're in a economy this, as it becomes more specialized, you're sort of losing the person who, like I said, just wants to work and go home. And so, or just like the general worker, like everyone wants, I have, I'm hiring for this position and this person needs to do this task. So I want someone who's done it for 10 years already. And it's like, it's a super specific task that you would only ever do on this team. It's like, have you considered just hiring someone with good traits and good experience and teaching them it?
+Jordan: Yeah, it feels like that's what companies used to do. Entry level like those entry level jobs don't exist basically like there if you go if you go to LinkedIn and you go to any entry level job you're gonna see they're required three to. Five years of experience. And it's like she said in the movie, she's like, if I don't have experience, how do I get experience? It's like, that's what it's like. I don't, it's bad.
+Darius: Well, you know, we're always chasing the ghost of 08. What else you got for act two?
+Jordan: Right. Okay, so they kind of, they're down bad. I don't know why that was funny to me. Whether they're down bad.
+Darius: Yeah. It's like selling *** didn't work.
+Jordan: So start scamming. They walk so Karisha could run. Pretty much.
+Darius: That's what I thought about that song too. She's definitely a child of this movie. So yes.
+Jordan: Yeah. So they kind of built this scheme to pick guys up at bars. drug them and then bring them to the strip club. They're not knowing if they worked there, I guess, as like ringers pretty much. Although I will say that the scene of them like cooking the **** was kind of crazy because how do you learn how to do that? And then also, if you're going to do that, why not just sell drugs? I don't know.
+Darius: You learn how to do that working in a strip club, which I'm sure it just like has drugs flowing in and out of it constantly. Well, Why not sell drugs? Honestly, I think a lot of them didn't see themselves as criminals. Yeah, like they thought that they were just like ripping off rich people.
+Jordan: Yeah, I think they thought they were Robin Hood.
+Darius: Yeah, that's not what my one of my questions is was what they did immoral. But clearly we both agree that drugging and bankrupting people who it's like, do they think that they were like, The CEO was in there. Like you're doing like mid managers like this. Like these are people with just like regular jobs within the organization of the bank. Like they're well paid, but they're not running a business.
+Jordan: The guys who are wealthy enough or have as much wealth as the girls thought they had, game would just hire hookers, I feel like. So.
+Darius: And it's just, yeah. The older me definitely views them a bit more critically than 2019 me did because yeah, they really like that guy's call. He's like, do I can't pay my mortgage?
+Jordan: I can't pay him work, dude. And they were maxing out everybody's cars.
+Darius: Yes. And company cars. People lost their jobs like your company credit card. Yeah. What are you going to tell them? Oh, I went to a strip club and they got robbed that you think your boss is going to hear that **** or believe you? It's just, you know, and I'm like, these aren't people who were tricking on you and got overboard. These are people you get robbed.
+Jordan: It's a totally different thing. Yeah, and I remember Cardi B, was stripping. She said she used to drug and rob guys. She said she used to do that **** to guys. And I remember people were like, yeah, well, they were going to abuse her anyway.
+Darius: And it's like, no, that's not how it works.
+Jordan: I don't know if that's how that works. Number one, #2, if you went to that guy's house and there was an agreement of services that were possibly going to be rendered, that's not.
+Darius: The same thing, She was dead wrong for trying to, I mean, just speaking of it so matter of factly, like just drugging people. Don't do that. Bad, bad Cardi. No, I don't think that they didn't want to do drugs. They didn't want to sell drugs because what they thought they were doing was like, you said, some sort of Robin Hood, some sort of benevolent activity when really what they were doing was, I mean, like multiple felonies. I'm surprised. In fact, they only went down for financial crimes. It's kind of wild because they were assaulting people.
+Jordan: Honestly, they got off really, really light. I don't know if it's because of the, they were women or if it's because of women.
+Darius: No, it's because they were women.
+Jordan: The time they were in or whatever. I don't know, maybe laws weren't strange, laws weren't stringent in 13, 2013. I don't know.
+Darius: Even the reception of this movie where it was, it was almost like joyous. I promise you a movie about a bunch of men drugging women would not be received as well.
+Jordan: Yes, absolutely right. Yes. Like imagine that scene where they throw the naked guy on the ground outside the hospital. Let's just swap all those roles.
+Darius: Yeah, I just.
+Jordan: What would we call that movie?
+Darius: I remember the energy around this movie. And it was it was very much not very much not. It was not it wasn't there was not a critical no analysis of the behavior. I'll put it that way.
+Jordan: Yeah. They treated it, what it was? It was almost treated like it was like John Q for moms.
+Darius: Yeah.
+Jordan: Like, the kid needed a new heart, so we had to rob the hospital.
+Darius: Yeah. That is interesting that I didn't think about it when I was watching this, but the reception of this movie was definitely not viewed through, we'll just call it like a Me Too lens, like it would have been if the gender roles were reversed.
+Jordan: Yes. Very true.
+Darius: What else you got for act 2?
+Jordan: Okay, so where do you think they went and left? I mean, obviously working with the cokehead chick was crazy, but do you think it was more so them leaving the club and trying to go independent, so to speak, with their little ring?
+Darius: I think like most people who commit financial crimes, They just, they went to the, where did they go left? I think they went left. I don't think there was ever a way to, sooner or later, they're gonna get caught. Someone's going to not care about being embarrassed to admit what happened to them. And they're gonna, you know, like I want, like, okay, I'll just, okay, I was, fell too hard for some women who were probably too hot for me, but they robbed me and I want justice for that. And that person's gonna have all the evidence and you're gonna go down. And they had, like I'm sure they started with, 100 bucks. But then when you're maxing out thousands of dollars, sooner or later, you're going to reach a point where someone just does not care to be embarrassed. They want revenge or justice or whatever you call it. So where they went left was going to the well one too many times. But I think that almost always happens with financial crimes. Ponzi schemes don't start as people trying to defraud people. They start with I promised this return and I can't get it, but I can go get a new investor and pay this person back. But by the time I flip the third one, I can pay everybody back.
+Jordan: I got to get another one.
+Darius: And then it works. Then you go and do it, usually you try to do it again. And then, you know, it eventually, and you keep, and it just, it never feels, you know, it's like addiction. People don't, I mean, outside of Mel on Snowfall, people don't become Rockheads overnight. It's always, you know, you go to the well, First it starts as a social thing and then it's a stressful thing. And then it's that. No one starts. She again, except for her. No one becomes a crackhead overnight. You know, it's a gradual thing. It's a party thing. Yeah. We're in the back room at a club and okay, I'm going to, you know, and then it's now you're now you're, you know, selling your microwave. Yeah. So it's It happens gradually then all at once is what they say.
+Jordan: Yeah. Do you think, I mean, Jayla's scared to kind of mention it a little bit, you know, well, she more so mentioned it in the long terms of the guys that wanted to get caught for like cheating or whatever. But do you think they factored into the, they took into account the fact that like men are less likely to report crimes against them?
+Darius: Yeah, for sure.
+Jordan: Things of that nature.
+Darius: The skeleton key of the whole thing was that they were women.
+Jordan: Yeah.
+Darius: You know, I the Weaponizing the power of male *****. Right. You know, I, it's like I've seen men willing to walk across hot coals barefoot to get, you know, to *** ****. It's so, and so that, and you know, they're pretty women, so they're harmless. And then the cops, how long did the cops hang up on people calling to try to report them? Right. it's just the entire premise of this was them believing that no one would take male victims seriously. Yeah. Yes.
+Jordan: Do you? Okay, so it might be for actor. I don't know. So there's a portion of interview where she, you can almost hear Constance Wu's character like bargaining almost like an addict where she's like, no, you have to understand like, We didn't think we were doing anything wrong. We're like, you have to understand these were guys who, would have, co</t>
   </si>
 </sst>
 </file>
@@ -7346,7 +7530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
@@ -8087,6 +8271,23 @@
         <v>68</v>
       </c>
     </row>
+    <row r="38" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" s="4">
+        <v>2019</v>
+      </c>
+      <c r="C38" s="7">
+        <v>4</v>
+      </c>
+      <c r="D38" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
@@ -8099,7 +8300,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5993E05E-2F2C-4E78-8DF8-86474A36DE5C}">
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
@@ -8399,6 +8600,14 @@
         <v>109</v>
       </c>
     </row>
+    <row r="38" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>